<commit_message>
Remove outdated contract files and update existing contracts with new details, including the addition of UBI custody fees for various agreements. Ensure all documents reflect accurate financial terms and maintain consistency across the archive.
</commit_message>
<xml_diff>
--- a/Dépenses/dépenses seb.xlsx
+++ b/Dépenses/dépenses seb.xlsx
@@ -1,32 +1,43 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29929"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30026"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://kheopst-my.sharepoint.com/personal/sebastien_dury_kheops_ch/Documents/PERSO/GN/2026/Dépenses/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="14" documentId="11_AD4DB114E441178AC67DF47D5E92E3C8683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{2610B597-837C-4ECF-A4D0-4AEF452F7922}"/>
+  <xr:revisionPtr revIDLastSave="18" documentId="11_AD4DB114E441178AC67DF47D5E92E3C8683EDF18" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{088BCB90-9CD8-41E1-ACE3-6B057763EF74}"/>
   <bookViews>
-    <workbookView minimized="1" xWindow="4320" yWindow="4290" windowWidth="21600" windowHeight="11295" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="765" windowWidth="28800" windowHeight="15435" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Tabelle1" sheetId="1" r:id="rId1"/>
     <sheet name="Sheet1" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
   <si>
     <t>gn celtiana Krondaar 2026</t>
   </si>
@@ -41,6 +52,9 @@
   </si>
   <si>
     <t>fumigènes vets (16)</t>
+  </si>
+  <si>
+    <t>tentures</t>
   </si>
 </sst>
 </file>
@@ -133,6 +147,50 @@
         <a:xfrm>
           <a:off x="1219200" y="952500"/>
           <a:ext cx="9107171" cy="4048690"/>
+        </a:xfrm>
+        <a:prstGeom prst="rect">
+          <a:avLst/>
+        </a:prstGeom>
+      </xdr:spPr>
+    </xdr:pic>
+    <xdr:clientData/>
+  </xdr:twoCellAnchor>
+  <xdr:twoCellAnchor editAs="oneCell">
+    <xdr:from>
+      <xdr:col>2</xdr:col>
+      <xdr:colOff>0</xdr:colOff>
+      <xdr:row>30</xdr:row>
+      <xdr:rowOff>0</xdr:rowOff>
+    </xdr:from>
+    <xdr:to>
+      <xdr:col>12</xdr:col>
+      <xdr:colOff>313524</xdr:colOff>
+      <xdr:row>50</xdr:row>
+      <xdr:rowOff>28095</xdr:rowOff>
+    </xdr:to>
+    <xdr:pic>
+      <xdr:nvPicPr>
+        <xdr:cNvPr id="3" name="Picture 2">
+          <a:extLst>
+            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{14D5D3A3-D84A-31A5-F48F-090D91A1F293}"/>
+            </a:ext>
+          </a:extLst>
+        </xdr:cNvPr>
+        <xdr:cNvPicPr>
+          <a:picLocks noChangeAspect="1"/>
+        </xdr:cNvPicPr>
+      </xdr:nvPicPr>
+      <xdr:blipFill>
+        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId2"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </xdr:blipFill>
+      <xdr:spPr>
+        <a:xfrm>
+          <a:off x="1219200" y="5715000"/>
+          <a:ext cx="6409524" cy="3838095"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -407,7 +465,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="C4:F10"/>
+  <dimension ref="C4:F14"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData>
     <row r="4" spans="3:6" x14ac:dyDescent="0.25">
@@ -445,6 +503,20 @@
       </c>
       <c r="F10">
         <v>65.48</v>
+      </c>
+    </row>
+    <row r="11" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="C11" t="s">
+        <v>5</v>
+      </c>
+      <c r="F11">
+        <v>142.41999999999999</v>
+      </c>
+    </row>
+    <row r="14" spans="3:6" x14ac:dyDescent="0.25">
+      <c r="F14">
+        <f>SUM(F7:F13)</f>
+        <v>545.22</v>
       </c>
     </row>
   </sheetData>

</xml_diff>